<commit_message>
atualizando script e incluindo grafico
</commit_message>
<xml_diff>
--- a/DATA/Classes de Uso do solo e Cobertura Vegetal - RJ.xlsx
+++ b/DATA/Classes de Uso do solo e Cobertura Vegetal - RJ.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Pós-doc\Disciplina R\Material Tidyverse + Ggplot\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\melis\OneDrive\Escritorio\areas-naturales\DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72576AA6-E3C9-4503-A774-D27121836396}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC019E84-6C83-47E8-B948-A7405FF04560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="269" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="269" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dados" sheetId="5" r:id="rId1"/>
@@ -32,6 +32,9 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -1020,9 +1023,6 @@
     <t>Área de Planejamento (AP)</t>
   </si>
   <si>
-    <t>Região de Planejamento (RP)</t>
-  </si>
-  <si>
     <t>Região Administrativa (RA)</t>
   </si>
   <si>
@@ -1054,6 +1054,9 @@
   </si>
   <si>
     <t xml:space="preserve">Maré </t>
+  </si>
+  <si>
+    <t>RP</t>
   </si>
 </sst>
 </file>
@@ -1263,9 +1266,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1303,9 +1306,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1338,9 +1341,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1373,9 +1393,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1550,7 +1587,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T175"/>
-  <sheetFormatPr defaultColWidth="14.6640625" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.6640625" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.6640625" style="2" customWidth="1"/>
     <col min="2" max="2" width="10" style="2" customWidth="1"/>
@@ -1571,10 +1608,10 @@
         <v>249</v>
       </c>
       <c r="C1" s="19" t="s">
+        <v>261</v>
+      </c>
+      <c r="D1" s="19" t="s">
         <v>250</v>
-      </c>
-      <c r="D1" s="19" t="s">
-        <v>251</v>
       </c>
       <c r="E1" s="20" t="s">
         <v>152</v>
@@ -1636,7 +1673,7 @@
         <v>247</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E2" s="17">
         <v>0</v>
@@ -1698,7 +1735,7 @@
         <v>247</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E3" s="17">
         <v>0</v>
@@ -1760,7 +1797,7 @@
         <v>247</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E4" s="17">
         <v>0</v>
@@ -1822,7 +1859,7 @@
         <v>247</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E5" s="17">
         <v>0</v>
@@ -2256,7 +2293,7 @@
         <v>247</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E12" s="17">
         <v>0</v>
@@ -2318,7 +2355,7 @@
         <v>247</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E13" s="17">
         <v>0</v>
@@ -2380,7 +2417,7 @@
         <v>247</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E14" s="17">
         <v>0</v>
@@ -2442,7 +2479,7 @@
         <v>247</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E15" s="17">
         <v>0</v>
@@ -2504,7 +2541,7 @@
         <v>247</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E16" s="5">
         <v>0</v>
@@ -2625,7 +2662,7 @@
         <v>2</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>15</v>
@@ -2687,7 +2724,7 @@
         <v>2</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>15</v>
@@ -2749,7 +2786,7 @@
         <v>2</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D20" s="7" t="s">
         <v>15</v>
@@ -2811,7 +2848,7 @@
         <v>2</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D21" s="7" t="s">
         <v>15</v>
@@ -2873,7 +2910,7 @@
         <v>2</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D22" s="7" t="s">
         <v>15</v>
@@ -2935,7 +2972,7 @@
         <v>2</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D23" s="7" t="s">
         <v>15</v>
@@ -2997,7 +3034,7 @@
         <v>2</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D24" s="7" t="s">
         <v>15</v>
@@ -3059,7 +3096,7 @@
         <v>2</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D25" s="7" t="s">
         <v>15</v>
@@ -3121,7 +3158,7 @@
         <v>2</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>23</v>
@@ -3183,7 +3220,7 @@
         <v>2</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>23</v>
@@ -3245,7 +3282,7 @@
         <v>2</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>27</v>
@@ -3307,7 +3344,7 @@
         <v>2</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>27</v>
@@ -3369,7 +3406,7 @@
         <v>2</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>27</v>
@@ -3431,7 +3468,7 @@
         <v>2</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>27</v>
@@ -3493,7 +3530,7 @@
         <v>2</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>27</v>
@@ -3555,7 +3592,7 @@
         <v>2</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>27</v>
@@ -3617,7 +3654,7 @@
         <v>2</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>27</v>
@@ -3679,10 +3716,10 @@
         <v>2</v>
       </c>
       <c r="C35" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="D35" s="3" t="s">
         <v>255</v>
-      </c>
-      <c r="D35" s="3" t="s">
-        <v>256</v>
       </c>
       <c r="E35" s="5">
         <v>0</v>
@@ -4417,7 +4454,7 @@
     </row>
     <row r="47" spans="1:20" s="3" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B47" s="3">
         <v>3</v>
@@ -4426,7 +4463,7 @@
         <v>138</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E47" s="5">
         <v>0</v>
@@ -5471,7 +5508,7 @@
     </row>
     <row r="64" spans="1:20" s="3" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B64" s="3">
         <v>3</v>
@@ -5480,7 +5517,7 @@
         <v>43</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E64" s="5">
         <v>0</v>
@@ -8205,10 +8242,10 @@
         <v>3</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D108" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E108" s="5">
         <v>0</v>
@@ -8267,10 +8304,10 @@
         <v>3</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D109" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E109" s="5">
         <v>0</v>
@@ -8329,10 +8366,10 @@
         <v>3</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D110" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E110" s="5">
         <v>0</v>
@@ -8391,10 +8428,10 @@
         <v>3</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D111" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E111" s="5">
         <v>0</v>
@@ -8453,10 +8490,10 @@
         <v>3</v>
       </c>
       <c r="C112" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D112" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E112" s="5">
         <v>0</v>
@@ -8515,10 +8552,10 @@
         <v>3</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D113" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E113" s="5">
         <v>0</v>
@@ -8577,10 +8614,10 @@
         <v>3</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D114" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E114" s="5">
         <v>0</v>
@@ -8639,10 +8676,10 @@
         <v>3</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D115" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E115" s="5">
         <v>0</v>
@@ -8701,10 +8738,10 @@
         <v>3</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D116" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E116" s="5">
         <v>0</v>
@@ -8763,10 +8800,10 @@
         <v>3</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D117" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E117" s="5">
         <v>0</v>
@@ -8825,10 +8862,10 @@
         <v>3</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D118" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E118" s="5">
         <v>0</v>
@@ -8887,10 +8924,10 @@
         <v>3</v>
       </c>
       <c r="C119" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D119" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E119" s="5">
         <v>0</v>
@@ -8949,10 +8986,10 @@
         <v>3</v>
       </c>
       <c r="C120" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D120" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E120" s="5">
         <v>0</v>
@@ -9011,10 +9048,10 @@
         <v>3</v>
       </c>
       <c r="C121" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D121" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E121" s="5">
         <v>0</v>
@@ -9073,10 +9110,10 @@
         <v>3</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D122" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E122" s="5">
         <v>0</v>
@@ -11695,7 +11732,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G80"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.109375" style="13" customWidth="1"/>
     <col min="2" max="7" width="9.109375" style="15" customWidth="1"/>

</xml_diff>